<commit_message>
Fix django-storages version requirement in requirements.txt to >=1.14.0
</commit_message>
<xml_diff>
--- a/selenium_tests/reports/test_analysis_report.xlsx
+++ b/selenium_tests/reports/test_analysis_report.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="98">
   <si>
     <t>NEXOLITH CARE - E2E TEST ANALYSIS REPORT</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Test Execution Timestamp</t>
   </si>
   <si>
-    <t>2026-08-22T09:09:18.993Z</t>
+    <t>2026-08-24T04:06:42.212Z</t>
   </si>
   <si>
     <t>Automated Run</t>
@@ -69,22 +69,22 @@
     <t>Failed Tests</t>
   </si>
   <si>
-    <t>Zero Errors</t>
+    <t>Action Required</t>
   </si>
   <si>
     <t>Pass Rate (%)</t>
   </si>
   <si>
-    <t>100%</t>
-  </si>
-  <si>
-    <t>HEALTHY</t>
+    <t>43%</t>
+  </si>
+  <si>
+    <t>DEGRADED</t>
   </si>
   <si>
     <t>Total Test Duration (sec)</t>
   </si>
   <si>
-    <t>10.61s</t>
+    <t>71.19s</t>
   </si>
   <si>
     <t>Performance Nominal</t>
@@ -177,10 +177,10 @@
     <t>Authentication Suite</t>
   </si>
   <si>
-    <t>User Account Registration &amp; JWT Generation</t>
-  </si>
-  <si>
-    <t>[data-testid="auth-submit"]</t>
+    <t>User Account Registration &amp; Email OTP Dispatch</t>
+  </si>
+  <si>
+    <t>[data-testid="register-submit"]</t>
   </si>
   <si>
     <t>TC-03</t>
@@ -189,7 +189,14 @@
     <t>User Login &amp; JWT Session Validation</t>
   </si>
   <si>
-    <t>[data-testid="username-input"]</t>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>[data-testid="login-username"]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for URL to contain "/dashboard"
+Wait timed out after 15184ms</t>
   </si>
   <si>
     <t>TC-04</t>
@@ -204,6 +211,10 @@
     <t>[data-testid="dashboard-container"]</t>
   </si>
   <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, [data-testid="dashboard-container"])
+Wait timed out after 15033ms</t>
+  </si>
+  <si>
     <t>TC-05</t>
   </si>
   <si>
@@ -216,6 +227,10 @@
     <t>[data-testid="report-file-input"]</t>
   </si>
   <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, [data-testid="report-file-input"])
+Wait timed out after 15020ms</t>
+  </si>
+  <si>
     <t>TC-06</t>
   </si>
   <si>
@@ -238,6 +253,10 @@
   </si>
   <si>
     <t>[data-testid="assistant-chat-input"]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, [data-testid="assistant-chat-input"])
+Wait timed out after 15039ms</t>
   </si>
   <si>
     <t>Component / Endpoint</t>
@@ -298,7 +317,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -320,7 +339,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="15803D"/>
+      <color rgb="B91C1C"/>
     </font>
     <font>
       <b/>
@@ -328,8 +347,14 @@
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="B91C1C"/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -351,6 +376,11 @@
         <fgColor rgb="DCFCE7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FEE2E2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -364,7 +394,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -377,6 +407,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -802,7 +835,7 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C9" t="s">
         <v>16</v>
@@ -813,7 +846,7 @@
         <v>17</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C10" t="s">
         <v>18</v>
@@ -956,7 +989,7 @@
         <v>49</v>
       </c>
       <c r="E2">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F2" t="s">
         <v>50</v>
@@ -979,7 +1012,7 @@
         <v>49</v>
       </c>
       <c r="E3">
-        <v>1794</v>
+        <v>4438</v>
       </c>
       <c r="F3" t="s">
         <v>55</v>
@@ -998,83 +1031,83 @@
       <c r="C4" t="s">
         <v>57</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>49</v>
+      <c r="D4" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="E4">
-        <v>675</v>
+        <v>15559</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G4" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>49</v>
+        <v>63</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="E5">
-        <v>138</v>
+        <v>15147</v>
       </c>
       <c r="F5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G5" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C6" t="s">
-        <v>65</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>49</v>
+        <v>68</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="E6">
-        <v>1169</v>
+        <v>15126</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G6" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C7" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>49</v>
       </c>
       <c r="E7">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G7" t="s">
         <v>51</v>
@@ -1082,25 +1115,25 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C8" t="s">
-        <v>73</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>49</v>
+        <v>77</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="E8">
-        <v>1845</v>
+        <v>15207</v>
       </c>
       <c r="F8" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G8" t="s">
-        <v>51</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1122,27 +1155,27 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>49</v>
@@ -1150,13 +1183,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>49</v>
@@ -1164,13 +1197,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>49</v>
@@ -1178,13 +1211,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>49</v>
@@ -1192,13 +1225,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C6" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>49</v>
@@ -1206,13 +1239,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>49</v>
@@ -1220,13 +1253,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C8" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>49</v>

</xml_diff>